<commit_message>
working through the buttons
</commit_message>
<xml_diff>
--- a/Wiring/RaspberryPinLayout.xlsx
+++ b/Wiring/RaspberryPinLayout.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01bcc1a4e60e225b/Active Folder/Programming/PycharmProjects/Stereotaxiccontrol/Wiring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{08C0758F-095E-44EE-8951-BCC9659F0E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{08C0758F-095E-44EE-8951-BCC9659F0E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{170A273B-2348-49A8-95D8-204557173501}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7ECF0DEC-3A74-4BBF-A655-3F5550588827}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{7ECF0DEC-3A74-4BBF-A655-3F5550588827}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="StereoPylot SR" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="46">
   <si>
     <t>Raspberry PI Pin Layout</t>
   </si>
@@ -144,6 +145,36 @@
   </si>
   <si>
     <t>Encoder Board GND</t>
+  </si>
+  <si>
+    <t>LimitGND</t>
+  </si>
+  <si>
+    <t>Limit AUX</t>
+  </si>
+  <si>
+    <t>hardwiredbutton-1</t>
+  </si>
+  <si>
+    <t>harwiredbutton -2</t>
+  </si>
+  <si>
+    <t>fourthRotoB</t>
+  </si>
+  <si>
+    <t>fourthRotoA</t>
+  </si>
+  <si>
+    <t>fourth step</t>
+  </si>
+  <si>
+    <t>fourth dir</t>
+  </si>
+  <si>
+    <t>harwiredbutton -3</t>
+  </si>
+  <si>
+    <t>hardwiredbutton-4</t>
   </si>
 </sst>
 </file>
@@ -542,11 +573,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530A0C4E-B887-428F-BA4A-B8D168D00CCA}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="11.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="29.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
+    <col min="3" max="5" width="11.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -627,7 +662,7 @@
         <v>3</v>
       </c>
       <c r="C7" s="2">
-        <f t="shared" ref="C7:D27" si="0">C6+2</f>
+        <f t="shared" ref="C7:D18" si="0">C6+2</f>
         <v>5</v>
       </c>
       <c r="D7" s="2">
@@ -867,11 +902,11 @@
         <v>5</v>
       </c>
       <c r="C19" s="2">
-        <f t="shared" ref="C19:C26" si="1">C18+2</f>
+        <f t="shared" ref="C19:C24" si="1">C18+2</f>
         <v>29</v>
       </c>
       <c r="D19" s="2">
-        <f t="shared" ref="D19:D26" si="2">D18+2</f>
+        <f t="shared" ref="D19:D24" si="2">D18+2</f>
         <v>30</v>
       </c>
       <c r="E19" s="1" t="s">
@@ -976,6 +1011,475 @@
       </c>
       <c r="D24" s="2">
         <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="E24" s="1">
+        <v>21</v>
+      </c>
+      <c r="F24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="96" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15E8BBD3-141B-414D-957B-63A3A174D36F}">
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
+    <col min="3" max="5" width="11.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2">
+        <f>C5+2</f>
+        <v>3</v>
+      </c>
+      <c r="D6" s="2">
+        <f>D5+2</f>
+        <v>4</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2">
+        <f t="shared" ref="C7:D22" si="0">C6+2</f>
+        <v>5</v>
+      </c>
+      <c r="D7" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D8" s="2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="E8" s="1">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="D9" s="2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E9" s="1">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1">
+        <v>17</v>
+      </c>
+      <c r="C10" s="2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="D10" s="2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="E10" s="1">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="D11" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="1">
+        <v>22</v>
+      </c>
+      <c r="C12" s="2">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="E12" s="1">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="2">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="D13" s="2">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="E13" s="1">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="1">
+        <v>10</v>
+      </c>
+      <c r="C14" s="2">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="D14" s="2">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1">
+        <v>9</v>
+      </c>
+      <c r="C15" s="2">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="D15" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="E15" s="1">
+        <v>25</v>
+      </c>
+      <c r="F15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="1">
+        <v>11</v>
+      </c>
+      <c r="C16" s="2">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="D16" s="2">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="E16" s="1">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="D17" s="2">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="E17" s="1">
+        <v>7</v>
+      </c>
+      <c r="F17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="2">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="D18" s="2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="1">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="D19" s="2">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="1">
+        <v>6</v>
+      </c>
+      <c r="C20" s="2">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="D20" s="2">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="E20" s="1">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="1">
+        <v>13</v>
+      </c>
+      <c r="C21" s="2">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="D21" s="2">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <v>19</v>
+      </c>
+      <c r="C22" s="2">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="D22" s="2">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="E22" s="1">
+        <v>16</v>
+      </c>
+      <c r="F22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="1">
+        <v>26</v>
+      </c>
+      <c r="C23" s="2">
+        <f t="shared" ref="C23:D24" si="1">C22+2</f>
+        <v>37</v>
+      </c>
+      <c r="D23" s="2">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="E23" s="1">
+        <v>20</v>
+      </c>
+      <c r="F23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2">
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="E24" s="1">

</xml_diff>

<commit_message>
testing rotaryclass timer funtion changes - test-steppersV4
</commit_message>
<xml_diff>
--- a/Wiring/RaspberryPinLayout.xlsx
+++ b/Wiring/RaspberryPinLayout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01bcc1a4e60e225b/Active Folder/Programming/PycharmProjects/Stereotaxiccontrol/Wiring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{08C0758F-095E-44EE-8951-BCC9659F0E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{170A273B-2348-49A8-95D8-204557173501}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{08C0758F-095E-44EE-8951-BCC9659F0E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD4B326F-676C-4BDA-ADA8-1E9E3FAC1AF6}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{7ECF0DEC-3A74-4BBF-A655-3F5550588827}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="76">
   <si>
     <t>Raspberry PI Pin Layout</t>
   </si>
@@ -175,6 +175,96 @@
   </si>
   <si>
     <t>hardwiredbutton-4</t>
+  </si>
+  <si>
+    <t>dvinsert</t>
+  </si>
+  <si>
+    <t>syring withdraw</t>
+  </si>
+  <si>
+    <t>fullretract</t>
+  </si>
+  <si>
+    <t>rezero</t>
+  </si>
+  <si>
+    <t>relzeroup5</t>
+  </si>
+  <si>
+    <t>rezerodvabs</t>
+  </si>
+  <si>
+    <t>abszero</t>
+  </si>
+  <si>
+    <t>presetpos</t>
+  </si>
+  <si>
+    <t>makeit</t>
+  </si>
+  <si>
+    <t>engage</t>
+  </si>
+  <si>
+    <t>down</t>
+  </si>
+  <si>
+    <t>up</t>
+  </si>
+  <si>
+    <t>apretract</t>
+  </si>
+  <si>
+    <t>apretur</t>
+  </si>
+  <si>
+    <t>fbregma</t>
+  </si>
+  <si>
+    <t>lambda</t>
+  </si>
+  <si>
+    <t>rat</t>
+  </si>
+  <si>
+    <t>mouse</t>
+  </si>
+  <si>
+    <t>function1</t>
+  </si>
+  <si>
+    <t>arm</t>
+  </si>
+  <si>
+    <t>zeroml</t>
+  </si>
+  <si>
+    <t>dvretract</t>
+  </si>
+  <si>
+    <t>dvreturn</t>
+  </si>
+  <si>
+    <t>zeroap</t>
+  </si>
+  <si>
+    <t>zeroall</t>
+  </si>
+  <si>
+    <t>probe</t>
+  </si>
+  <si>
+    <t>drill</t>
+  </si>
+  <si>
+    <t>coaese&gt;</t>
+  </si>
+  <si>
+    <t>fine</t>
+  </si>
+  <si>
+    <t>zerodv</t>
   </si>
 </sst>
 </file>
@@ -207,12 +297,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -227,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -239,6 +335,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1028,7 +1125,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15E8BBD3-141B-414D-957B-63A3A174D36F}">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.88671875" customWidth="1"/>
@@ -1037,17 +1134,37 @@
     <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I1">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1066,8 +1183,14 @@
       <c r="F4" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1086,8 +1209,14 @@
       <c r="F5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1105,8 +1234,14 @@
       <c r="E6" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1127,8 +1262,14 @@
       <c r="F7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I7">
+        <v>6</v>
+      </c>
+      <c r="J7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1149,8 +1290,14 @@
       <c r="F8" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I8">
+        <v>7</v>
+      </c>
+      <c r="J8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
@@ -1168,8 +1315,14 @@
       <c r="F9" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I9">
+        <v>8</v>
+      </c>
+      <c r="J9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -1190,8 +1343,14 @@
       <c r="F10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I10">
+        <v>9</v>
+      </c>
+      <c r="J10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -1212,8 +1371,14 @@
       <c r="F11" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I11">
+        <v>10</v>
+      </c>
+      <c r="J11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1234,8 +1399,14 @@
       <c r="F12" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I12">
+        <v>11</v>
+      </c>
+      <c r="J12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>5</v>
       </c>
@@ -1253,8 +1424,14 @@
       <c r="F13" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I13">
+        <v>12</v>
+      </c>
+      <c r="J13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1275,8 +1452,14 @@
       <c r="F14" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I14">
+        <v>13</v>
+      </c>
+      <c r="J14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1297,8 +1480,14 @@
       <c r="F15" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I15">
+        <v>14</v>
+      </c>
+      <c r="J15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -1319,8 +1508,14 @@
       <c r="F16" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I16">
+        <v>15</v>
+      </c>
+      <c r="J16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -1341,8 +1536,14 @@
       <c r="F17" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I17">
+        <v>16</v>
+      </c>
+      <c r="J17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -1363,8 +1564,14 @@
       <c r="F18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I18">
+        <v>17</v>
+      </c>
+      <c r="J18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1382,8 +1589,14 @@
       <c r="E19" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I19">
+        <v>18</v>
+      </c>
+      <c r="J19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -1404,8 +1617,14 @@
       <c r="F20" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I20">
+        <v>19</v>
+      </c>
+      <c r="J20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -1423,8 +1642,14 @@
       <c r="E21" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I21">
+        <v>20</v>
+      </c>
+      <c r="J21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1445,8 +1670,14 @@
       <c r="F22" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I22">
+        <v>21</v>
+      </c>
+      <c r="J22" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -1467,8 +1698,14 @@
       <c r="F23" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I23">
+        <v>22</v>
+      </c>
+      <c r="J23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -1487,6 +1724,70 @@
       </c>
       <c r="F24" t="s">
         <v>33</v>
+      </c>
+      <c r="I24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I25">
+        <v>24</v>
+      </c>
+      <c r="J25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I26">
+        <v>25</v>
+      </c>
+      <c r="J26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I27">
+        <v>26</v>
+      </c>
+      <c r="J27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I28">
+        <v>27</v>
+      </c>
+      <c r="J28" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I29">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I30">
+        <v>29</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I31">
+        <v>30</v>
+      </c>
+      <c r="J31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I32">
+        <v>31</v>
+      </c>
+      <c r="J32" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating the right hand to PCB
</commit_message>
<xml_diff>
--- a/Wiring/RaspberryPinLayout.xlsx
+++ b/Wiring/RaspberryPinLayout.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01bcc1a4e60e225b/Active Folder/Programming/PycharmProjects/Stereotaxiccontrol/Wiring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{08C0758F-095E-44EE-8951-BCC9659F0E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{08C0758F-095E-44EE-8951-BCC9659F0E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB37C4C5-B07E-4CA5-9748-5D9E79728E4B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7ECF0DEC-3A74-4BBF-A655-3F5550588827}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{7ECF0DEC-3A74-4BBF-A655-3F5550588827}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="StereoPylot SR" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="85">
   <si>
     <t>Raspberry PI Pin Layout</t>
   </si>
@@ -144,6 +146,153 @@
   </si>
   <si>
     <t>Encoder Board GND</t>
+  </si>
+  <si>
+    <t>LimitGND</t>
+  </si>
+  <si>
+    <t>Limit AUX</t>
+  </si>
+  <si>
+    <t>hardwiredbutton-1</t>
+  </si>
+  <si>
+    <t>harwiredbutton -2</t>
+  </si>
+  <si>
+    <t>fourthRotoB</t>
+  </si>
+  <si>
+    <t>fourthRotoA</t>
+  </si>
+  <si>
+    <t>fourth step</t>
+  </si>
+  <si>
+    <t>fourth dir</t>
+  </si>
+  <si>
+    <t>harwiredbutton -3</t>
+  </si>
+  <si>
+    <t>hardwiredbutton-4</t>
+  </si>
+  <si>
+    <t>dvinsert</t>
+  </si>
+  <si>
+    <t>syring withdraw</t>
+  </si>
+  <si>
+    <t>fullretract</t>
+  </si>
+  <si>
+    <t>rezero</t>
+  </si>
+  <si>
+    <t>relzeroup5</t>
+  </si>
+  <si>
+    <t>rezerodvabs</t>
+  </si>
+  <si>
+    <t>abszero</t>
+  </si>
+  <si>
+    <t>presetpos</t>
+  </si>
+  <si>
+    <t>makeit</t>
+  </si>
+  <si>
+    <t>engage</t>
+  </si>
+  <si>
+    <t>down</t>
+  </si>
+  <si>
+    <t>up</t>
+  </si>
+  <si>
+    <t>apretract</t>
+  </si>
+  <si>
+    <t>apretur</t>
+  </si>
+  <si>
+    <t>fbregma</t>
+  </si>
+  <si>
+    <t>lambda</t>
+  </si>
+  <si>
+    <t>rat</t>
+  </si>
+  <si>
+    <t>mouse</t>
+  </si>
+  <si>
+    <t>function1</t>
+  </si>
+  <si>
+    <t>arm</t>
+  </si>
+  <si>
+    <t>zeroml</t>
+  </si>
+  <si>
+    <t>dvretract</t>
+  </si>
+  <si>
+    <t>dvreturn</t>
+  </si>
+  <si>
+    <t>zeroap</t>
+  </si>
+  <si>
+    <t>zeroall</t>
+  </si>
+  <si>
+    <t>probe</t>
+  </si>
+  <si>
+    <t>drill</t>
+  </si>
+  <si>
+    <t>coaese&gt;</t>
+  </si>
+  <si>
+    <t>fine</t>
+  </si>
+  <si>
+    <t>zerodv</t>
+  </si>
+  <si>
+    <t>DV is AP encoder</t>
+  </si>
+  <si>
+    <t>AP is DV encoder</t>
+  </si>
+  <si>
+    <t>AP backwards</t>
+  </si>
+  <si>
+    <t>Speed fine</t>
+  </si>
+  <si>
+    <t>DV motor get warm</t>
+  </si>
+  <si>
+    <t>ML motor gets warm</t>
+  </si>
+  <si>
+    <t>Speed Med</t>
+  </si>
+  <si>
+    <t>Speed Coarse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">relactiveDV button not registering in program - works for the test-buttons </t>
   </si>
 </sst>
 </file>
@@ -176,12 +325,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -196,7 +351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -208,6 +363,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -542,11 +698,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530A0C4E-B887-428F-BA4A-B8D168D00CCA}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="11.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="29.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
+    <col min="3" max="5" width="11.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -627,7 +787,7 @@
         <v>3</v>
       </c>
       <c r="C7" s="2">
-        <f t="shared" ref="C7:D27" si="0">C6+2</f>
+        <f t="shared" ref="C7:D18" si="0">C6+2</f>
         <v>5</v>
       </c>
       <c r="D7" s="2">
@@ -867,11 +1027,11 @@
         <v>5</v>
       </c>
       <c r="C19" s="2">
-        <f t="shared" ref="C19:C26" si="1">C18+2</f>
+        <f t="shared" ref="C19:C24" si="1">C18+2</f>
         <v>29</v>
       </c>
       <c r="D19" s="2">
-        <f t="shared" ref="D19:D26" si="2">D18+2</f>
+        <f t="shared" ref="D19:D24" si="2">D18+2</f>
         <v>30</v>
       </c>
       <c r="E19" s="1" t="s">
@@ -983,6 +1143,728 @@
       </c>
       <c r="F24" t="s">
         <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="96" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15E8BBD3-141B-414D-957B-63A3A174D36F}">
+  <dimension ref="A1:J32"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
+    <col min="3" max="5" width="11.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2">
+        <f>C5+2</f>
+        <v>3</v>
+      </c>
+      <c r="D6" s="2">
+        <f>D5+2</f>
+        <v>4</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2">
+        <f t="shared" ref="C7:D22" si="0">C6+2</f>
+        <v>5</v>
+      </c>
+      <c r="D7" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
+      <c r="J7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D8" s="2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="E8" s="1">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>41</v>
+      </c>
+      <c r="I8">
+        <v>7</v>
+      </c>
+      <c r="J8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="D9" s="2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E9" s="1">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9">
+        <v>8</v>
+      </c>
+      <c r="J9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1">
+        <v>17</v>
+      </c>
+      <c r="C10" s="2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="D10" s="2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="E10" s="1">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10">
+        <v>9</v>
+      </c>
+      <c r="J10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="D11" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11">
+        <v>10</v>
+      </c>
+      <c r="J11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="1">
+        <v>22</v>
+      </c>
+      <c r="C12" s="2">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="E12" s="1">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12">
+        <v>11</v>
+      </c>
+      <c r="J12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="2">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="D13" s="2">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="E13" s="1">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13">
+        <v>12</v>
+      </c>
+      <c r="J13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="1">
+        <v>10</v>
+      </c>
+      <c r="C14" s="2">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="D14" s="2">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
+      <c r="J14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1">
+        <v>9</v>
+      </c>
+      <c r="C15" s="2">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="D15" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="E15" s="1">
+        <v>25</v>
+      </c>
+      <c r="F15" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15">
+        <v>14</v>
+      </c>
+      <c r="J15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="1">
+        <v>11</v>
+      </c>
+      <c r="C16" s="2">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="D16" s="2">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="E16" s="1">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>29</v>
+      </c>
+      <c r="I16">
+        <v>15</v>
+      </c>
+      <c r="J16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="D17" s="2">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="E17" s="1">
+        <v>7</v>
+      </c>
+      <c r="F17" t="s">
+        <v>42</v>
+      </c>
+      <c r="I17">
+        <v>16</v>
+      </c>
+      <c r="J17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="2">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="D18" s="2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
+        <v>43</v>
+      </c>
+      <c r="I18">
+        <v>17</v>
+      </c>
+      <c r="J18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="1">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="D19" s="2">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I19">
+        <v>18</v>
+      </c>
+      <c r="J19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="1">
+        <v>6</v>
+      </c>
+      <c r="C20" s="2">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="D20" s="2">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="E20" s="1">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
+        <v>30</v>
+      </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
+      <c r="J20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="1">
+        <v>13</v>
+      </c>
+      <c r="C21" s="2">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="D21" s="2">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I21">
+        <v>20</v>
+      </c>
+      <c r="J21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1">
+        <v>19</v>
+      </c>
+      <c r="C22" s="2">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="D22" s="2">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="E22" s="1">
+        <v>16</v>
+      </c>
+      <c r="F22" t="s">
+        <v>31</v>
+      </c>
+      <c r="I22">
+        <v>21</v>
+      </c>
+      <c r="J22" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="1">
+        <v>26</v>
+      </c>
+      <c r="C23" s="2">
+        <f t="shared" ref="C23:D24" si="1">C22+2</f>
+        <v>37</v>
+      </c>
+      <c r="D23" s="2">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="E23" s="1">
+        <v>20</v>
+      </c>
+      <c r="F23" t="s">
+        <v>32</v>
+      </c>
+      <c r="I23">
+        <v>22</v>
+      </c>
+      <c r="J23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="E24" s="1">
+        <v>21</v>
+      </c>
+      <c r="F24" t="s">
+        <v>33</v>
+      </c>
+      <c r="I24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I25">
+        <v>24</v>
+      </c>
+      <c r="J25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I26">
+        <v>25</v>
+      </c>
+      <c r="J26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I27">
+        <v>26</v>
+      </c>
+      <c r="J27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I28">
+        <v>27</v>
+      </c>
+      <c r="J28" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I29">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I30">
+        <v>29</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I31">
+        <v>30</v>
+      </c>
+      <c r="J31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I32">
+        <v>31</v>
+      </c>
+      <c r="J32" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9ABA796-617F-4C03-913E-9AD2E7D1581B}">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>